<commit_message>
fix bird data to use schema image
</commit_message>
<xml_diff>
--- a/test_data/birds/data/additional-ro-crate-metadata.xlsx
+++ b/test_data/birds/data/additional-ro-crate-metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bbb/sandbox/casey-ro-crate-html-lite/ro-crate-html-lite/test_data/birds/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bbb/sandbox/ro-crate-static-site/test_data/birds/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B498A2E-3344-E446-B2E4-D77B3973741C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314C9C66-4A59-0A45-BE2A-32C01278ED0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="32440" windowHeight="18160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RootDataset" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="77">
   <si>
     <t>name</t>
   </si>
@@ -104,9 +104,6 @@
     <t>custom:scientificName</t>
   </si>
   <si>
-    <t>isRef_custom:image</t>
-  </si>
-  <si>
     <t>isRef_custom:callAudio</t>
   </si>
   <si>
@@ -161,15 +158,6 @@
     <t>the translation of this entry's story</t>
   </si>
   <si>
-    <t>arcp://name,custom/terms#image</t>
-  </si>
-  <si>
-    <t>image</t>
-  </si>
-  <si>
-    <t>the bird image</t>
-  </si>
-  <si>
     <t>callAudio</t>
   </si>
   <si>
@@ -279,6 +267,9 @@
   </si>
   <si>
     <t>about them</t>
+  </si>
+  <si>
+    <t>isRef_image</t>
   </si>
 </sst>
 </file>
@@ -707,7 +698,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -715,7 +706,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -797,7 +788,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>6</v>
@@ -824,22 +815,22 @@
         <v>19</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>20</v>
       </c>
       <c r="O1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="16" x14ac:dyDescent="0.2">
@@ -848,10 +839,10 @@
         <v>#magpie</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E2" s="5" t="str">
         <f>K2</f>
@@ -861,40 +852,40 @@
         <v>3</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="K2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -920,52 +911,52 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -1280,10 +1271,10 @@
         <v>#person_1</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1319,128 +1310,114 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
         <v>30</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>31</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>32</v>
-      </c>
-      <c r="D2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="B3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>35</v>
-      </c>
-      <c r="D3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
         <v>37</v>
       </c>
-      <c r="B4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>38</v>
-      </c>
-      <c r="D4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1465,21 +1442,21 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
         <v>3</v>

</xml_diff>